<commit_message>
updated code and ata
</commit_message>
<xml_diff>
--- a/example_david.xlsx
+++ b/example_david.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,6 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$A$1:$R$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet3!$A$1:$W$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$A$1:$R$1</definedName>
   </definedNames>
   <calcPr/>
@@ -1958,6 +1959,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" min="3" max="3" width="10.61328125"/>
+  </cols>
   <sheetData>
     <row r="1" ht="28.5">
       <c r="A1" s="1" t="s">
@@ -4375,6 +4379,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:W1"/>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>